<commit_message>
Adding more BBC site data
</commit_message>
<xml_diff>
--- a/raw_data/age_sex_named_subjects.xlsx
+++ b/raw_data/age_sex_named_subjects.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/8099077b681ff7d8/Documents/A - UniKonstanz/Thesis/Capuchin_HC_foraging_efficiency_and_selectivity/raw_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{56112C07-952E-46B1-817F-A8EEFE27D34D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="8_{56112C07-952E-46B1-817F-A8EEFE27D34D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{691C703F-48BF-4FD0-858A-CC33B0011D70}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{4D44F5B2-B406-4CE5-BE6B-7416F5D6CCF7}"/>
+    <workbookView xWindow="4305" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{4D44F5B2-B406-4CE5-BE6B-7416F5D6CCF7}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="198" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="210" uniqueCount="72">
   <si>
     <t>T</t>
   </si>
@@ -243,6 +243,18 @@
   </si>
   <si>
     <t>adut male</t>
+  </si>
+  <si>
+    <t>Adult Male</t>
+  </si>
+  <si>
+    <t>Fuji</t>
+  </si>
+  <si>
+    <t>Caesar</t>
+  </si>
+  <si>
+    <t>Wayne</t>
   </si>
 </sst>
 </file>
@@ -633,7 +645,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F7191118-2807-40F8-9DE6-19E177A1BEC5}">
-  <dimension ref="A1:F39"/>
+  <dimension ref="A1:F42"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="14.26953125" customWidth="1"/>
@@ -1315,6 +1327,48 @@
         <v>61</v>
       </c>
     </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A40" t="s">
+        <v>47</v>
+      </c>
+      <c r="B40" t="s">
+        <v>69</v>
+      </c>
+      <c r="C40" t="s">
+        <v>52</v>
+      </c>
+      <c r="D40" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A41" t="s">
+        <v>47</v>
+      </c>
+      <c r="B41" t="s">
+        <v>70</v>
+      </c>
+      <c r="C41" t="s">
+        <v>52</v>
+      </c>
+      <c r="D41" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A42" t="s">
+        <v>47</v>
+      </c>
+      <c r="B42" t="s">
+        <v>71</v>
+      </c>
+      <c r="C42" t="s">
+        <v>52</v>
+      </c>
+      <c r="D42" t="s">
+        <v>68</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Annotating and adding to bernoulli models Updating subjects age/sex class
</commit_message>
<xml_diff>
--- a/raw_data/age_sex_named_subjects.xlsx
+++ b/raw_data/age_sex_named_subjects.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/8099077b681ff7d8/Documents/A - UniKonstanz/Thesis/Capuchin_HC_foraging_efficiency_and_selectivity/raw_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3" documentId="8_{56112C07-952E-46B1-817F-A8EEFE27D34D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{691C703F-48BF-4FD0-858A-CC33B0011D70}"/>
+  <xr:revisionPtr revIDLastSave="12" documentId="8_{56112C07-952E-46B1-817F-A8EEFE27D34D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BF9D60B1-37EF-4978-B68E-F5B54FC21AEB}"/>
   <bookViews>
-    <workbookView xWindow="4305" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{4D44F5B2-B406-4CE5-BE6B-7416F5D6CCF7}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{4D44F5B2-B406-4CE5-BE6B-7416F5D6CCF7}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="210" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="259" uniqueCount="74">
   <si>
     <t>T</t>
   </si>
@@ -242,12 +242,6 @@
     <t>juvenile male</t>
   </si>
   <si>
-    <t>adut male</t>
-  </si>
-  <si>
-    <t>Adult Male</t>
-  </si>
-  <si>
     <t>Fuji</t>
   </si>
   <si>
@@ -255,6 +249,18 @@
   </si>
   <si>
     <t>Wayne</t>
+  </si>
+  <si>
+    <t>Brendan</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Still need ID matched </t>
+  </si>
+  <si>
+    <t>Maybe</t>
+  </si>
+  <si>
+    <t>asubadult male</t>
   </si>
 </sst>
 </file>
@@ -326,6 +332,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -645,7 +655,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F7191118-2807-40F8-9DE6-19E177A1BEC5}">
-  <dimension ref="A1:F42"/>
+  <dimension ref="A1:G42"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="14.26953125" customWidth="1"/>
@@ -1086,6 +1096,12 @@
       <c r="D22" t="s">
         <v>61</v>
       </c>
+      <c r="E22" t="s">
+        <v>3</v>
+      </c>
+      <c r="F22" t="s">
+        <v>70</v>
+      </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
@@ -1100,6 +1116,12 @@
       <c r="D23" t="s">
         <v>62</v>
       </c>
+      <c r="E23" t="s">
+        <v>3</v>
+      </c>
+      <c r="F23" t="s">
+        <v>70</v>
+      </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
@@ -1114,6 +1136,12 @@
       <c r="D24" t="s">
         <v>66</v>
       </c>
+      <c r="E24" t="s">
+        <v>3</v>
+      </c>
+      <c r="F24" t="s">
+        <v>70</v>
+      </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
@@ -1128,6 +1156,12 @@
       <c r="D25" t="s">
         <v>66</v>
       </c>
+      <c r="E25" t="s">
+        <v>3</v>
+      </c>
+      <c r="F25" t="s">
+        <v>70</v>
+      </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
@@ -1142,6 +1176,12 @@
       <c r="D26" t="s">
         <v>64</v>
       </c>
+      <c r="E26" t="s">
+        <v>3</v>
+      </c>
+      <c r="F26" t="s">
+        <v>70</v>
+      </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
@@ -1154,7 +1194,13 @@
         <v>38</v>
       </c>
       <c r="D27" t="s">
-        <v>64</v>
+        <v>62</v>
+      </c>
+      <c r="E27" t="s">
+        <v>3</v>
+      </c>
+      <c r="F27" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.35">
@@ -1170,6 +1216,12 @@
       <c r="D28" t="s">
         <v>62</v>
       </c>
+      <c r="E28" t="s">
+        <v>3</v>
+      </c>
+      <c r="F28" t="s">
+        <v>70</v>
+      </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
@@ -1184,6 +1236,12 @@
       <c r="D29" t="s">
         <v>61</v>
       </c>
+      <c r="E29" t="s">
+        <v>3</v>
+      </c>
+      <c r="F29" t="s">
+        <v>70</v>
+      </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
@@ -1198,6 +1256,12 @@
       <c r="D30" t="s">
         <v>62</v>
       </c>
+      <c r="E30" t="s">
+        <v>3</v>
+      </c>
+      <c r="F30" t="s">
+        <v>70</v>
+      </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
@@ -1210,7 +1274,13 @@
         <v>31</v>
       </c>
       <c r="D31" t="s">
-        <v>67</v>
+        <v>62</v>
+      </c>
+      <c r="E31" t="s">
+        <v>3</v>
+      </c>
+      <c r="F31" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.35">
@@ -1226,8 +1296,14 @@
       <c r="D32" t="s">
         <v>66</v>
       </c>
-    </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="E32" t="s">
+        <v>3</v>
+      </c>
+      <c r="F32" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>29</v>
       </c>
@@ -1240,8 +1316,14 @@
       <c r="D33" t="s">
         <v>66</v>
       </c>
-    </row>
-    <row r="34" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="E33" t="s">
+        <v>3</v>
+      </c>
+      <c r="F33" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A34" s="2" t="s">
         <v>29</v>
       </c>
@@ -1254,10 +1336,14 @@
       <c r="D34" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="E34" s="2"/>
-      <c r="F34" s="2"/>
-    </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="E34" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="F34" s="2" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>47</v>
       </c>
@@ -1270,8 +1356,17 @@
       <c r="D35" t="s">
         <v>66</v>
       </c>
-    </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="E35" t="s">
+        <v>3</v>
+      </c>
+      <c r="F35" t="s">
+        <v>70</v>
+      </c>
+      <c r="G35" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>47</v>
       </c>
@@ -1284,8 +1379,17 @@
       <c r="D36" t="s">
         <v>66</v>
       </c>
-    </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="E36" t="s">
+        <v>3</v>
+      </c>
+      <c r="F36" t="s">
+        <v>70</v>
+      </c>
+      <c r="G36" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>47</v>
       </c>
@@ -1298,8 +1402,14 @@
       <c r="D37" t="s">
         <v>61</v>
       </c>
-    </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="E37" t="s">
+        <v>3</v>
+      </c>
+      <c r="F37" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>47</v>
       </c>
@@ -1312,8 +1422,17 @@
       <c r="D38" t="s">
         <v>66</v>
       </c>
-    </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="E38" t="s">
+        <v>3</v>
+      </c>
+      <c r="F38" t="s">
+        <v>70</v>
+      </c>
+      <c r="G38" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>47</v>
       </c>
@@ -1324,49 +1443,85 @@
         <v>52</v>
       </c>
       <c r="D39" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.35">
+        <v>62</v>
+      </c>
+      <c r="E39" t="s">
+        <v>72</v>
+      </c>
+      <c r="F39" t="s">
+        <v>70</v>
+      </c>
+      <c r="G39" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>47</v>
       </c>
       <c r="B40" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="C40" t="s">
         <v>52</v>
       </c>
       <c r="D40" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.35">
+        <v>73</v>
+      </c>
+      <c r="E40" t="s">
+        <v>72</v>
+      </c>
+      <c r="F40" t="s">
+        <v>70</v>
+      </c>
+      <c r="G40" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>47</v>
       </c>
       <c r="B41" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="C41" t="s">
         <v>52</v>
       </c>
       <c r="D41" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.35">
+        <v>61</v>
+      </c>
+      <c r="E41" t="s">
+        <v>3</v>
+      </c>
+      <c r="F41" t="s">
+        <v>70</v>
+      </c>
+      <c r="G41" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>47</v>
       </c>
       <c r="B42" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C42" t="s">
         <v>52</v>
       </c>
       <c r="D42" t="s">
-        <v>68</v>
+        <v>61</v>
+      </c>
+      <c r="E42" t="s">
+        <v>72</v>
+      </c>
+      <c r="F42" t="s">
+        <v>70</v>
+      </c>
+      <c r="G42" t="s">
+        <v>71</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Adding age-sex to ellipse plot
</commit_message>
<xml_diff>
--- a/raw_data/age_sex_named_subjects.xlsx
+++ b/raw_data/age_sex_named_subjects.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/8099077b681ff7d8/Documents/A - UniKonstanz/Thesis/Capuchin_HC_foraging_efficiency_and_selectivity/raw_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="12" documentId="8_{56112C07-952E-46B1-817F-A8EEFE27D34D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BF9D60B1-37EF-4978-B68E-F5B54FC21AEB}"/>
+  <xr:revisionPtr revIDLastSave="13" documentId="8_{56112C07-952E-46B1-817F-A8EEFE27D34D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{39600F1C-5E22-452F-A23F-DF225B5A9090}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{4D44F5B2-B406-4CE5-BE6B-7416F5D6CCF7}"/>
+    <workbookView xWindow="4305" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{4D44F5B2-B406-4CE5-BE6B-7416F5D6CCF7}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="259" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="259" uniqueCount="73">
   <si>
     <t>T</t>
   </si>
@@ -258,9 +258,6 @@
   </si>
   <si>
     <t>Maybe</t>
-  </si>
-  <si>
-    <t>asubadult male</t>
   </si>
 </sst>
 </file>
@@ -1466,7 +1463,7 @@
         <v>52</v>
       </c>
       <c r="D40" t="s">
-        <v>73</v>
+        <v>62</v>
       </c>
       <c r="E40" t="s">
         <v>72</v>

</xml_diff>

<commit_message>
Adjusting so that age and sex also have separate columns per individual
</commit_message>
<xml_diff>
--- a/raw_data/age_sex_named_subjects.xlsx
+++ b/raw_data/age_sex_named_subjects.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/8099077b681ff7d8/Documents/A - UniKonstanz/Thesis/Capuchin_HC_foraging_efficiency_and_selectivity/raw_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="13" documentId="8_{56112C07-952E-46B1-817F-A8EEFE27D34D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{39600F1C-5E22-452F-A23F-DF225B5A9090}"/>
+  <xr:revisionPtr revIDLastSave="123" documentId="8_{56112C07-952E-46B1-817F-A8EEFE27D34D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3141CE1B-92DE-4226-B3BC-E0332960EA02}"/>
   <bookViews>
-    <workbookView xWindow="4305" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{4D44F5B2-B406-4CE5-BE6B-7416F5D6CCF7}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{4D44F5B2-B406-4CE5-BE6B-7416F5D6CCF7}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="259" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="356" uniqueCount="84">
   <si>
     <t>T</t>
   </si>
@@ -258,6 +258,39 @@
   </si>
   <si>
     <t>Maybe</t>
+  </si>
+  <si>
+    <t>age</t>
+  </si>
+  <si>
+    <t>sex</t>
+  </si>
+  <si>
+    <t>adult</t>
+  </si>
+  <si>
+    <t>subadult</t>
+  </si>
+  <si>
+    <t>juvenile</t>
+  </si>
+  <si>
+    <t>Balthasar</t>
+  </si>
+  <si>
+    <t>Doodle</t>
+  </si>
+  <si>
+    <t>JUV; Named individual from BBC Stream</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>male</t>
+  </si>
+  <si>
+    <t>female</t>
   </si>
 </sst>
 </file>
@@ -310,10 +343,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -652,15 +689,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F7191118-2807-40F8-9DE6-19E177A1BEC5}">
-  <dimension ref="A1:G42"/>
+  <dimension ref="A1:I44"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="14.26953125" customWidth="1"/>
     <col min="3" max="3" width="48.54296875" customWidth="1"/>
-    <col min="4" max="4" width="16.7265625" customWidth="1"/>
+    <col min="4" max="6" width="16.7265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>56</v>
       </c>
@@ -674,13 +711,19 @@
         <v>58</v>
       </c>
       <c r="E1" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="G1" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -694,13 +737,19 @@
         <v>61</v>
       </c>
       <c r="E2" t="s">
-        <v>3</v>
+        <v>75</v>
       </c>
       <c r="F2" t="s">
+        <v>82</v>
+      </c>
+      <c r="G2" t="s">
+        <v>3</v>
+      </c>
+      <c r="H2" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>0</v>
       </c>
@@ -714,13 +763,19 @@
         <v>61</v>
       </c>
       <c r="E3" t="s">
-        <v>3</v>
+        <v>75</v>
       </c>
       <c r="F3" t="s">
+        <v>82</v>
+      </c>
+      <c r="G3" t="s">
+        <v>3</v>
+      </c>
+      <c r="H3" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>0</v>
       </c>
@@ -734,13 +789,19 @@
         <v>62</v>
       </c>
       <c r="E4" t="s">
-        <v>3</v>
+        <v>76</v>
       </c>
       <c r="F4" t="s">
+        <v>82</v>
+      </c>
+      <c r="G4" t="s">
+        <v>3</v>
+      </c>
+      <c r="H4" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>0</v>
       </c>
@@ -754,13 +815,19 @@
         <v>63</v>
       </c>
       <c r="E5" t="s">
-        <v>3</v>
+        <v>76</v>
       </c>
       <c r="F5" t="s">
+        <v>83</v>
+      </c>
+      <c r="G5" t="s">
+        <v>3</v>
+      </c>
+      <c r="H5" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>0</v>
       </c>
@@ -774,13 +841,19 @@
         <v>61</v>
       </c>
       <c r="E6" t="s">
-        <v>3</v>
+        <v>75</v>
       </c>
       <c r="F6" t="s">
+        <v>82</v>
+      </c>
+      <c r="G6" t="s">
+        <v>3</v>
+      </c>
+      <c r="H6" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>0</v>
       </c>
@@ -794,13 +867,19 @@
         <v>61</v>
       </c>
       <c r="E7" t="s">
-        <v>3</v>
+        <v>75</v>
       </c>
       <c r="F7" t="s">
+        <v>82</v>
+      </c>
+      <c r="G7" t="s">
+        <v>3</v>
+      </c>
+      <c r="H7" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>0</v>
       </c>
@@ -814,13 +893,19 @@
         <v>61</v>
       </c>
       <c r="E8" t="s">
-        <v>3</v>
+        <v>75</v>
       </c>
       <c r="F8" t="s">
+        <v>82</v>
+      </c>
+      <c r="G8" t="s">
+        <v>3</v>
+      </c>
+      <c r="H8" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>0</v>
       </c>
@@ -834,13 +919,19 @@
         <v>62</v>
       </c>
       <c r="E9" t="s">
-        <v>3</v>
+        <v>76</v>
       </c>
       <c r="F9" t="s">
+        <v>82</v>
+      </c>
+      <c r="G9" t="s">
+        <v>3</v>
+      </c>
+      <c r="H9" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>0</v>
       </c>
@@ -854,13 +945,19 @@
         <v>63</v>
       </c>
       <c r="E10" t="s">
-        <v>3</v>
+        <v>76</v>
       </c>
       <c r="F10" t="s">
+        <v>83</v>
+      </c>
+      <c r="G10" t="s">
+        <v>3</v>
+      </c>
+      <c r="H10" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>0</v>
       </c>
@@ -874,13 +971,19 @@
         <v>64</v>
       </c>
       <c r="E11" t="s">
-        <v>3</v>
+        <v>75</v>
       </c>
       <c r="F11" t="s">
+        <v>83</v>
+      </c>
+      <c r="G11" t="s">
+        <v>3</v>
+      </c>
+      <c r="H11" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>0</v>
       </c>
@@ -894,13 +997,19 @@
         <v>63</v>
       </c>
       <c r="E12" t="s">
-        <v>3</v>
+        <v>76</v>
       </c>
       <c r="F12" t="s">
+        <v>83</v>
+      </c>
+      <c r="G12" t="s">
+        <v>3</v>
+      </c>
+      <c r="H12" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>0</v>
       </c>
@@ -914,13 +1023,19 @@
         <v>61</v>
       </c>
       <c r="E13" t="s">
-        <v>3</v>
+        <v>75</v>
       </c>
       <c r="F13" t="s">
+        <v>82</v>
+      </c>
+      <c r="G13" t="s">
+        <v>3</v>
+      </c>
+      <c r="H13" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>0</v>
       </c>
@@ -934,13 +1049,19 @@
         <v>65</v>
       </c>
       <c r="E14" t="s">
-        <v>3</v>
+        <v>76</v>
       </c>
       <c r="F14" t="s">
+        <v>82</v>
+      </c>
+      <c r="G14" t="s">
+        <v>3</v>
+      </c>
+      <c r="H14" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>0</v>
       </c>
@@ -954,13 +1075,19 @@
         <v>66</v>
       </c>
       <c r="E15" t="s">
-        <v>3</v>
+        <v>77</v>
       </c>
       <c r="F15" t="s">
+        <v>82</v>
+      </c>
+      <c r="G15" t="s">
+        <v>3</v>
+      </c>
+      <c r="H15" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>0</v>
       </c>
@@ -974,13 +1101,19 @@
         <v>64</v>
       </c>
       <c r="E16" t="s">
-        <v>3</v>
+        <v>75</v>
       </c>
       <c r="F16" t="s">
+        <v>83</v>
+      </c>
+      <c r="G16" t="s">
+        <v>3</v>
+      </c>
+      <c r="H16" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>0</v>
       </c>
@@ -994,13 +1127,19 @@
         <v>64</v>
       </c>
       <c r="E17" t="s">
-        <v>3</v>
+        <v>75</v>
       </c>
       <c r="F17" t="s">
+        <v>83</v>
+      </c>
+      <c r="G17" t="s">
+        <v>3</v>
+      </c>
+      <c r="H17" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>0</v>
       </c>
@@ -1014,13 +1153,19 @@
         <v>64</v>
       </c>
       <c r="E18" t="s">
-        <v>3</v>
+        <v>75</v>
       </c>
       <c r="F18" t="s">
+        <v>83</v>
+      </c>
+      <c r="G18" t="s">
+        <v>3</v>
+      </c>
+      <c r="H18" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>0</v>
       </c>
@@ -1034,13 +1179,19 @@
         <v>64</v>
       </c>
       <c r="E19" t="s">
-        <v>3</v>
+        <v>75</v>
       </c>
       <c r="F19" t="s">
+        <v>83</v>
+      </c>
+      <c r="G19" t="s">
+        <v>3</v>
+      </c>
+      <c r="H19" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>0</v>
       </c>
@@ -1054,13 +1205,19 @@
         <v>64</v>
       </c>
       <c r="E20" t="s">
-        <v>3</v>
+        <v>75</v>
       </c>
       <c r="F20" t="s">
+        <v>83</v>
+      </c>
+      <c r="G20" t="s">
+        <v>3</v>
+      </c>
+      <c r="H20" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="21" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A21" s="2" t="s">
         <v>0</v>
       </c>
@@ -1074,13 +1231,19 @@
         <v>64</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>3</v>
+        <v>75</v>
       </c>
       <c r="F21" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="G21" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="H21" s="2" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>29</v>
       </c>
@@ -1093,14 +1256,20 @@
       <c r="D22" t="s">
         <v>61</v>
       </c>
-      <c r="E22" t="s">
-        <v>3</v>
+      <c r="E22" s="3" t="s">
+        <v>75</v>
       </c>
       <c r="F22" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
+        <v>82</v>
+      </c>
+      <c r="G22" t="s">
+        <v>3</v>
+      </c>
+      <c r="H22" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>29</v>
       </c>
@@ -1114,13 +1283,19 @@
         <v>62</v>
       </c>
       <c r="E23" t="s">
-        <v>3</v>
+        <v>76</v>
       </c>
       <c r="F23" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
+        <v>82</v>
+      </c>
+      <c r="G23" t="s">
+        <v>3</v>
+      </c>
+      <c r="H23" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>29</v>
       </c>
@@ -1134,13 +1309,19 @@
         <v>66</v>
       </c>
       <c r="E24" t="s">
-        <v>3</v>
+        <v>77</v>
       </c>
       <c r="F24" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
+        <v>82</v>
+      </c>
+      <c r="G24" t="s">
+        <v>3</v>
+      </c>
+      <c r="H24" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>29</v>
       </c>
@@ -1154,13 +1335,19 @@
         <v>66</v>
       </c>
       <c r="E25" t="s">
-        <v>3</v>
+        <v>77</v>
       </c>
       <c r="F25" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
+        <v>82</v>
+      </c>
+      <c r="G25" t="s">
+        <v>3</v>
+      </c>
+      <c r="H25" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>29</v>
       </c>
@@ -1174,13 +1361,19 @@
         <v>64</v>
       </c>
       <c r="E26" t="s">
-        <v>3</v>
+        <v>75</v>
       </c>
       <c r="F26" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
+        <v>83</v>
+      </c>
+      <c r="G26" t="s">
+        <v>3</v>
+      </c>
+      <c r="H26" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>29</v>
       </c>
@@ -1194,13 +1387,19 @@
         <v>62</v>
       </c>
       <c r="E27" t="s">
-        <v>3</v>
+        <v>76</v>
       </c>
       <c r="F27" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
+        <v>82</v>
+      </c>
+      <c r="G27" t="s">
+        <v>3</v>
+      </c>
+      <c r="H27" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>29</v>
       </c>
@@ -1214,13 +1413,19 @@
         <v>62</v>
       </c>
       <c r="E28" t="s">
-        <v>3</v>
+        <v>76</v>
       </c>
       <c r="F28" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
+        <v>82</v>
+      </c>
+      <c r="G28" t="s">
+        <v>3</v>
+      </c>
+      <c r="H28" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>29</v>
       </c>
@@ -1234,13 +1439,19 @@
         <v>61</v>
       </c>
       <c r="E29" t="s">
-        <v>3</v>
+        <v>75</v>
       </c>
       <c r="F29" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.35">
+        <v>82</v>
+      </c>
+      <c r="G29" t="s">
+        <v>3</v>
+      </c>
+      <c r="H29" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>29</v>
       </c>
@@ -1254,13 +1465,19 @@
         <v>62</v>
       </c>
       <c r="E30" t="s">
-        <v>3</v>
+        <v>76</v>
       </c>
       <c r="F30" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.35">
+        <v>82</v>
+      </c>
+      <c r="G30" t="s">
+        <v>3</v>
+      </c>
+      <c r="H30" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>29</v>
       </c>
@@ -1274,13 +1491,19 @@
         <v>62</v>
       </c>
       <c r="E31" t="s">
-        <v>3</v>
+        <v>76</v>
       </c>
       <c r="F31" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.35">
+        <v>82</v>
+      </c>
+      <c r="G31" t="s">
+        <v>3</v>
+      </c>
+      <c r="H31" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>29</v>
       </c>
@@ -1294,13 +1517,19 @@
         <v>66</v>
       </c>
       <c r="E32" t="s">
-        <v>3</v>
+        <v>77</v>
       </c>
       <c r="F32" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.35">
+        <v>82</v>
+      </c>
+      <c r="G32" t="s">
+        <v>3</v>
+      </c>
+      <c r="H32" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>29</v>
       </c>
@@ -1314,13 +1543,19 @@
         <v>66</v>
       </c>
       <c r="E33" t="s">
-        <v>3</v>
+        <v>77</v>
       </c>
       <c r="F33" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="34" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+        <v>82</v>
+      </c>
+      <c r="G33" t="s">
+        <v>3</v>
+      </c>
+      <c r="H33" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A34" s="2" t="s">
         <v>29</v>
       </c>
@@ -1334,13 +1569,19 @@
         <v>61</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>3</v>
+        <v>75</v>
       </c>
       <c r="F34" s="2" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.35">
+        <v>82</v>
+      </c>
+      <c r="G34" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="H34" s="2" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>47</v>
       </c>
@@ -1353,17 +1594,23 @@
       <c r="D35" t="s">
         <v>66</v>
       </c>
-      <c r="E35" t="s">
-        <v>3</v>
-      </c>
-      <c r="F35" t="s">
-        <v>70</v>
+      <c r="E35" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="F35" s="3" t="s">
+        <v>82</v>
       </c>
       <c r="G35" t="s">
+        <v>3</v>
+      </c>
+      <c r="H35" t="s">
+        <v>70</v>
+      </c>
+      <c r="I35" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>47</v>
       </c>
@@ -1377,16 +1624,22 @@
         <v>66</v>
       </c>
       <c r="E36" t="s">
-        <v>3</v>
-      </c>
-      <c r="F36" t="s">
-        <v>70</v>
+        <v>77</v>
+      </c>
+      <c r="F36" s="3" t="s">
+        <v>82</v>
       </c>
       <c r="G36" t="s">
+        <v>3</v>
+      </c>
+      <c r="H36" t="s">
+        <v>70</v>
+      </c>
+      <c r="I36" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>47</v>
       </c>
@@ -1400,13 +1653,19 @@
         <v>61</v>
       </c>
       <c r="E37" t="s">
-        <v>3</v>
-      </c>
-      <c r="F37" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.35">
+        <v>75</v>
+      </c>
+      <c r="F37" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="G37" t="s">
+        <v>3</v>
+      </c>
+      <c r="H37" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>47</v>
       </c>
@@ -1420,16 +1679,22 @@
         <v>66</v>
       </c>
       <c r="E38" t="s">
-        <v>3</v>
-      </c>
-      <c r="F38" t="s">
-        <v>70</v>
+        <v>77</v>
+      </c>
+      <c r="F38" s="3" t="s">
+        <v>82</v>
       </c>
       <c r="G38" t="s">
+        <v>3</v>
+      </c>
+      <c r="H38" t="s">
+        <v>70</v>
+      </c>
+      <c r="I38" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>47</v>
       </c>
@@ -1443,16 +1708,22 @@
         <v>62</v>
       </c>
       <c r="E39" t="s">
+        <v>76</v>
+      </c>
+      <c r="F39" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="G39" t="s">
         <v>72</v>
       </c>
-      <c r="F39" t="s">
-        <v>70</v>
-      </c>
-      <c r="G39" t="s">
+      <c r="H39" t="s">
+        <v>70</v>
+      </c>
+      <c r="I39" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>47</v>
       </c>
@@ -1466,16 +1737,22 @@
         <v>62</v>
       </c>
       <c r="E40" t="s">
+        <v>76</v>
+      </c>
+      <c r="F40" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="G40" t="s">
         <v>72</v>
       </c>
-      <c r="F40" t="s">
-        <v>70</v>
-      </c>
-      <c r="G40" t="s">
+      <c r="H40" t="s">
+        <v>70</v>
+      </c>
+      <c r="I40" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>47</v>
       </c>
@@ -1489,16 +1766,22 @@
         <v>61</v>
       </c>
       <c r="E41" t="s">
-        <v>3</v>
-      </c>
-      <c r="F41" t="s">
-        <v>70</v>
+        <v>75</v>
+      </c>
+      <c r="F41" s="3" t="s">
+        <v>82</v>
       </c>
       <c r="G41" t="s">
+        <v>3</v>
+      </c>
+      <c r="H41" t="s">
+        <v>70</v>
+      </c>
+      <c r="I41" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>47</v>
       </c>
@@ -1512,13 +1795,62 @@
         <v>61</v>
       </c>
       <c r="E42" t="s">
+        <v>75</v>
+      </c>
+      <c r="F42" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="G42" t="s">
         <v>72</v>
       </c>
-      <c r="F42" t="s">
-        <v>70</v>
-      </c>
-      <c r="G42" t="s">
+      <c r="H42" t="s">
+        <v>70</v>
+      </c>
+      <c r="I42" t="s">
         <v>71</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A43" t="s">
+        <v>47</v>
+      </c>
+      <c r="B43" t="s">
+        <v>78</v>
+      </c>
+      <c r="C43" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="D43" t="s">
+        <v>61</v>
+      </c>
+      <c r="E43" t="s">
+        <v>75</v>
+      </c>
+      <c r="F43" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="G43" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="44" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A44" t="s">
+        <v>47</v>
+      </c>
+      <c r="B44" t="s">
+        <v>79</v>
+      </c>
+      <c r="C44" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="D44" t="s">
+        <v>77</v>
+      </c>
+      <c r="E44" t="s">
+        <v>77</v>
+      </c>
+      <c r="G44" t="s">
+        <v>81</v>
       </c>
     </row>
   </sheetData>

</xml_diff>